<commit_message>
fix: make PHS6 package quantity explicit in Rev E BOM
</commit_message>
<xml_diff>
--- a/outputs/20261001_reve_bom_audit/2026_BIZ-Lab_재료비관리_RevE_검수수정.xlsx
+++ b/outputs/20261001_reve_bom_audit/2026_BIZ-Lab_재료비관리_RevE_검수수정.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" r:id="Rbae726872b1c47d2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" r:id="R5bd21c202001454a"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2142,7 +2142,7 @@
         <x:v>한국미스미</x:v>
       </x:c>
       <x:c r="D61" s="14" t="str">
-        <x:v>상부 로드엔드</x:v>
+        <x:v>상부 로드엔드 (PHS6 2개입/포장)</x:v>
       </x:c>
       <x:c r="E61" s="14" t="str">
         <x:v>280-7599 / PHS6</x:v>
@@ -2157,7 +2157,7 @@
         <x:v>26124</x:v>
       </x:c>
       <x:c r="I61" s="5" t="str">
-        <x:v>M03. VAT 포함 표시가를 공급가로 환산. 재고·배송비·최종 결제금액 확인.</x:v>
+        <x:v>M03. 수량 2포장×2개입=4개, 3축에 3개 사용·1개 잔여. 한국미스미 결제 화면에서 실제 포장 단위·재고·납기 재확인.</x:v>
       </x:c>
       <x:c r="M61" s="1"/>
     </x:row>
@@ -8881,75 +8881,75 @@
     </x:row>
   </x:sheetData>
   <x:hyperlinks>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G4" r:id="R4a8374201cdf48c4"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G5" r:id="R1e466180b3804d0f"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G6" r:id="R1c784f7fb20e4031"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G7" r:id="R3960c14bf0904ad2"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G8" r:id="R6c34f0113e2748c0"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G9" r:id="R3aae37b14c3745b3"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G10" r:id="Rc6514ba50b5a4e89"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G11" r:id="R27b11e1b690b4329"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G12" r:id="R32818c0026d747c8"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G13" r:id="R9b90f397452840cf"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G14" r:id="Refe18a854f1547c9"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G15" r:id="R45c76b5107394b36"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G16" r:id="R4f43d0b9cae14ba4"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G17" r:id="R3a74762e9a2d47ce"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G18" r:id="R253c5bf38e0f4760"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G19" r:id="Rcd97370e6ff941cf"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G20" r:id="R8399428832be4683"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G21" r:id="Rd392b1a2e0bb4f24"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G22" r:id="R629510da6a344fc7"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G23" r:id="R7982c7ad4c3c4b3d"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G24" r:id="Rbca5130b42734118"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G25" r:id="R0251dccf62694e2d"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G26" r:id="R2c76197e671343f8"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G27" r:id="R16381ef672b34180"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G28" r:id="R5eb1c421139e4ced"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G29" r:id="Rdc436581b47746f2"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G30" r:id="Racd73330a4404765"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G31" r:id="R23da61c9582b41e6"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G32" r:id="Rd528766dc7ce4ebf"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G33" r:id="R13da7aa109e84733"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G34" r:id="Re41742a672324b5e"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G35" r:id="Rea129ad02f0d453e"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G36" r:id="R26f40e420a3c4e9e"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G37" r:id="Rec55f3c3cc8b440b"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G38" r:id="R2948bcad5daf44fb"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G39" r:id="R10728dcb671f497e"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G40" r:id="R2e71ebb419a34967"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G41" r:id="R3dc3552e85fd4e95"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G42" r:id="Re1067719fb414421"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G43" r:id="R693ad0f84b174a93"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G44" r:id="R39b8711035a249ac"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G45" r:id="R26df53d4113d426c"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G46" r:id="Rd063efdccfc04615"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G47" r:id="R568373d6fd2147ed"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G48" r:id="Rdd37cd161cf24a0a"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G49" r:id="R787c888db8ad4431"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G50" r:id="R68fa60c8dbc54ab9"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G51" r:id="R49c35ef0902f4370"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G52" r:id="Rd3a5f9d882e34709"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G53" r:id="R8bd53b1ef8bd4223"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G54" r:id="Ra3a9f8569e1f4b62"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G55" r:id="Re1321882c7e34e29"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G56" r:id="R481dfaf06b384d0e"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G57" r:id="Rcd763abbe1b84c5a"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G58" r:id="Rf0af26acf70b4a40"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G59" r:id="Rd815cf4401bc4088"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G60" r:id="R98a62ffd2c7a476b"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G61" r:id="R035c7752f0454cf2"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G62" r:id="R4e2fcce5ff054cda"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G63" r:id="Rf6310a2155ac4864"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G64" r:id="Rdba0394435844ee5"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G65" r:id="Rf516c8161bbe4a13"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G66" r:id="R3cbdf9b1004e4213"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G67" r:id="R68c8fb8187ec48c2"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G4" r:id="Rc94bcf776b7949c6"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G5" r:id="R6aab61b457ea4c40"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G6" r:id="R3cb9db0d5bb9461a"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G7" r:id="R9cc14f6f2e9349e2"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G8" r:id="Rdc878a2f546b4402"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G9" r:id="R20e65afa92ef49a0"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G10" r:id="Rab354a8b0c7c4ed1"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G11" r:id="R56f927f83f6e41dd"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G12" r:id="Re16628436f5f4042"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G13" r:id="Ra87daf5932fa40b8"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G14" r:id="R3c4b1912c897466c"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G15" r:id="Rcd1065c0d76c42b1"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G16" r:id="R9106ee66f62c40b5"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G17" r:id="Rf504492d73d344b2"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G18" r:id="Raaeb2c78543f4948"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G19" r:id="Rb099782e73244c09"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G20" r:id="Rd0ed77b3260642fe"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G21" r:id="R7f8edffc27aa4516"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G22" r:id="R55d2c1edb9284b3d"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G23" r:id="R78998d9b6b2a4b2f"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G24" r:id="R7e2b2bac167348b0"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G25" r:id="R3471f857e93a414f"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G26" r:id="R14dade84cb324b8d"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G27" r:id="R4e232c3291c849f6"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G28" r:id="R5f7f4f0c0fb54385"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G29" r:id="R15f76ded8fab48f0"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G30" r:id="R8d21015dd819444e"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G31" r:id="Rad32a368ff6d47e6"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G32" r:id="R934348266853492e"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G33" r:id="R98ab74721f514855"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G34" r:id="Re646baac42314802"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G35" r:id="R8fc2f95b05f941ec"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G36" r:id="Rea37fc1ab4df4c65"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G37" r:id="R70049173fc1442f1"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G38" r:id="Rbb45eea12aba4c77"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G39" r:id="Rd33dca314caa4e0f"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G40" r:id="Rfe6aefe841344ac3"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G41" r:id="Rb57d99d4ac474727"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G42" r:id="Rf64d5365f2b04285"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G43" r:id="R29b62d037c264986"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G44" r:id="R0e2fde9e41914bc0"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G45" r:id="R8a6f7c1c240b4984"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G46" r:id="Rc2c8760718ee4052"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G47" r:id="Red864c4f27dd4612"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G48" r:id="R14bf999c7e0549b9"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G49" r:id="R95a4798291074feb"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G50" r:id="R6e3bc7c025c44568"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G51" r:id="R8264e72b01864b3c"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G52" r:id="R7f746086e9c9454d"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G53" r:id="R9d890a3a03d84536"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G54" r:id="Rc3bf21da6fb24482"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G55" r:id="Rdf529216bf0e4cbf"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G56" r:id="R6655e92469704159"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G57" r:id="R04068e482b2c45e0"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G58" r:id="R40408af56eda415b"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G59" r:id="Ra0603fa82f404dcc"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G60" r:id="Rce8d385bd33745fa"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G61" r:id="R77e76054c6ed44f7"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G62" r:id="R727e3bba0c5749a4"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G63" r:id="R4a398e02ed224b40"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G64" r:id="Rfae50000d1b24632"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G65" r:id="R50ed42ab9a2e40a4"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G66" r:id="R23d2c7d2f9d144cf"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G67" r:id="R9e7dd4a1a5694ad2"/>
     <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G68" r:id="rId1"/>
     <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G69" r:id="rId2"/>
     <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G70" r:id="rId3"/>
   </x:hyperlinks>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6f4b41f56f914186"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb66a9df849a34148"/>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Audit RevE power branching and correct held BOM price
</commit_message>
<xml_diff>
--- a/outputs/20261001_reve_bom_audit/2026_BIZ-Lab_재료비관리_RevE_검수수정.xlsx
+++ b/outputs/20261001_reve_bom_audit/2026_BIZ-Lab_재료비관리_RevE_검수수정.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" r:id="R5bd21c202001454a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" r:id="Rabbf533d5f7c401e"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -533,7 +533,7 @@
   <x:sheetData>
     <x:row r="1" s="13" customFormat="1" ht="16.5" customHeight="1">
       <x:c r="B1" s="23" t="str">
-        <x:v>검수용 · 발주 보류 (2026-10-01)</x:v>
+        <x:v>검수용 · 발주 보류 (2026-10-02)</x:v>
       </x:c>
       <x:c r="C1" s="1"/>
       <x:c r="D1" s="1"/>
@@ -1644,7 +1644,7 @@
         <x:v>2600</x:v>
       </x:c>
       <x:c r="I42" s="5" t="str">
-        <x:v>E13. Portenta START 입력용. 접촉기 코일은 E10 NC 직렬 회로로 제어.</x:v>
+        <x:v>E13. START 순간버튼. 기존 E-stop NC+G9EA 코일 직렬안은 해제만으로 재투입 위험. K1 자기유지·재시작 차단 회로 미확정.</x:v>
       </x:c>
       <x:c r="M42" s="1"/>
     </x:row>
@@ -1668,10 +1668,10 @@
         <x:v>https://www.devicemart.co.kr/goods/view?no=14981941</x:v>
       </x:c>
       <x:c r="H43" s="18" t="n">
-        <x:v>72000</x:v>
+        <x:v>82800</x:v>
       </x:c>
       <x:c r="I43" s="5" t="str">
-        <x:v>E14. M5 출력 허용 4–16 mm², 현 AWG14 분기선 약 2.08 mm² 불가. XK2 대체안은 입력 10 mm² 이상과 상류 분기 재설계 필요.</x:v>
+        <x:v>E14. 2026-10-02 디바이스마트 표시가 41,400원/개×2. 현 2개+14AWG 배선은 부적합. BPS 1개+DKD35 3개 후보는 아직 배선/함체 미승인. 그대로 주문 금지.</x:v>
       </x:c>
       <x:c r="M43" s="1"/>
     </x:row>
@@ -1698,7 +1698,7 @@
         <x:v>34400</x:v>
       </x:c>
       <x:c r="I44" s="5" t="str">
-        <x:v>E15. AWG8 약 8.37 mm²는 XK2 입력 최소 10 mm² 미달. G9EA 제조사 주접점 권장선 14–22 mm²에도 미달.</x:v>
+        <x:v>E15. 현 8AWG는 G9EA 권장 유연전선 14~22mm² 미달. 16SQ 주간선·색상·실제 길이·M5/M6 러그·압착 수단 미확정. 그대로 주문 금지.</x:v>
       </x:c>
       <x:c r="M44" s="1"/>
     </x:row>
@@ -1779,7 +1779,7 @@
         <x:v>1600</x:v>
       </x:c>
       <x:c r="I47" s="5" t="str">
-        <x:v>HP01. 현 링크 판매 최소수량 100개 단위, 기재수량·가격은 주문 불가. 공통선 규격 재결정 후 링 규격/압착 방법 재선정.</x:v>
+        <x:v>HP01. 현 8AWG/M6 부품은 재선정 대상이고 링크 최소 100개 단위. 16SQ/M6 2개 이상 소량구매 후보 확인 중. 그대로 주문 금지.</x:v>
       </x:c>
       <x:c r="M47" s="1"/>
     </x:row>
@@ -1914,7 +1914,7 @@
         <x:v>800</x:v>
       </x:c>
       <x:c r="I52" s="5" t="str">
-        <x:v>HP02. 현 링크 판매 최소수량 100개 단위, 기재수량·가격은 주문 불가. PSU/G9EA 단자와 전선 규격 확정 후 교체.</x:v>
+        <x:v>HP02. 현 8AWG/M5 부품은 재선정 대상이고 링크 최소 100개 단위. 검토용 16SQ 배선 토폴로지에는 M5 접점 7개이나 러그 외형/압착 미승인. 그대로 주문 금지.</x:v>
       </x:c>
       <x:c r="M52" s="1"/>
     </x:row>
@@ -1941,7 +1941,7 @@
         <x:v>600</x:v>
       </x:c>
       <x:c r="I53" s="5" t="str">
-        <x:v>HP03. 현 링크 판매 최소수량 100개 단위. BPS 출력 최소 4 mm²와 현 14AWG 단자는 불일치하므로 단순 증량 금지.</x:v>
+        <x:v>HP03. 현 BPS 출력 최소 4mm²에 14AWG 불가. DKD35 후보 채택 시 퓨즈홀더/단자 종단 방식으로 재선정. 링크 최소 100개 단위. 그대로 주문 금지.</x:v>
       </x:c>
       <x:c r="M53" s="1"/>
     </x:row>
@@ -2292,7 +2292,7 @@
         <x:v>600</x:v>
       </x:c>
       <x:c r="I66" s="5" t="str">
-        <x:v>F11. 미스미 M6×25 3개×200원(공급가). 명목 적층 25 mm가 정확히 소진되어 PHS 암나사 깊이·물림·공차 검증 전 사용 보류.</x:v>
+        <x:v>F11. F07 스프링너트 실제 두께 5mm. M6×25는 현 CAD 적층에서 명목 1mm 홈 아래 돌출. 홈바닥·컵포인트 유효 나사물림 미확정. 그대로 주문 금지.</x:v>
       </x:c>
       <x:c r="M66" s="1"/>
     </x:row>
@@ -2319,7 +2319,7 @@
         <x:v>248157</x:v>
       </x:c>
       <x:c r="I67" s="5" t="str">
-        <x:v>E11. G9EA-1-B DC24: 접점 M5, 코일 M3.5/약 208 mA, 장착 M6. 접점 극성 준수. Portenta J6 출력+E-stop NC 직렬 코일 경로; 실배선 검증.</x:v>
+        <x:v>E11. G9EA 주접점 극성 준수. Portenta J6+E-stop 직렬 코일 경로는 자동 재투입 위험으로 폐기. START+K1 자기유지, 코일 서지억제·재시작 차단 회로 미확정. 그대로 주문 금지.</x:v>
       </x:c>
       <x:c r="M67" s="1"/>
     </x:row>
@@ -2415,7 +2415,7 @@
       <x:c r="G71" s="6"/>
       <x:c r="H71" s="19" t="n">
         <x:f>SUM(H4:H70)</x:f>
-        <x:v>2846985</x:v>
+        <x:v>2857785</x:v>
       </x:c>
       <x:c r="I71" s="7"/>
       <x:c r="M71" s="1"/>
@@ -2431,7 +2431,7 @@
       <x:c r="G72"/>
       <x:c r="H72" t="n">
         <x:f>ROUND(H71*10%,0)</x:f>
-        <x:v>284699</x:v>
+        <x:v>285779</x:v>
       </x:c>
       <x:c r="I72"/>
       <x:c r="M72" s="1"/>
@@ -2447,7 +2447,7 @@
       <x:c r="G73"/>
       <x:c r="H73" t="n">
         <x:f>SUM(H71:H72)</x:f>
-        <x:v>3131684</x:v>
+        <x:v>3143564</x:v>
       </x:c>
       <x:c r="I73"/>
       <x:c r="M73" s="1"/>
@@ -2463,10 +2463,10 @@
       <x:c r="G74"/>
       <x:c r="H74" t="n">
         <x:f>$I$2-H73</x:f>
-        <x:v>868316</x:v>
+        <x:v>856436</x:v>
       </x:c>
       <x:c r="I74" t="str">
-        <x:v>미확정 비용 제외. 결제 금지.</x:v>
+        <x:v>미확정 비용 제외. E14 현재가 반영한 검수용 산술이며 현 BOM 그대로 결제 금지.</x:v>
       </x:c>
       <x:c r="M74" s="1"/>
     </x:row>
@@ -8881,75 +8881,75 @@
     </x:row>
   </x:sheetData>
   <x:hyperlinks>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G4" r:id="Rc94bcf776b7949c6"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G5" r:id="R6aab61b457ea4c40"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G6" r:id="R3cb9db0d5bb9461a"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G7" r:id="R9cc14f6f2e9349e2"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G8" r:id="Rdc878a2f546b4402"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G9" r:id="R20e65afa92ef49a0"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G10" r:id="Rab354a8b0c7c4ed1"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G11" r:id="R56f927f83f6e41dd"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G12" r:id="Re16628436f5f4042"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G13" r:id="Ra87daf5932fa40b8"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G14" r:id="R3c4b1912c897466c"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G15" r:id="Rcd1065c0d76c42b1"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G16" r:id="R9106ee66f62c40b5"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G17" r:id="Rf504492d73d344b2"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G18" r:id="Raaeb2c78543f4948"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G19" r:id="Rb099782e73244c09"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G20" r:id="Rd0ed77b3260642fe"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G21" r:id="R7f8edffc27aa4516"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G22" r:id="R55d2c1edb9284b3d"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G23" r:id="R78998d9b6b2a4b2f"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G24" r:id="R7e2b2bac167348b0"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G25" r:id="R3471f857e93a414f"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G26" r:id="R14dade84cb324b8d"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G27" r:id="R4e232c3291c849f6"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G28" r:id="R5f7f4f0c0fb54385"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G29" r:id="R15f76ded8fab48f0"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G30" r:id="R8d21015dd819444e"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G31" r:id="Rad32a368ff6d47e6"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G32" r:id="R934348266853492e"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G33" r:id="R98ab74721f514855"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G34" r:id="Re646baac42314802"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G35" r:id="R8fc2f95b05f941ec"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G36" r:id="Rea37fc1ab4df4c65"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G37" r:id="R70049173fc1442f1"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G38" r:id="Rbb45eea12aba4c77"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G39" r:id="Rd33dca314caa4e0f"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G40" r:id="Rfe6aefe841344ac3"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G41" r:id="Rb57d99d4ac474727"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G42" r:id="Rf64d5365f2b04285"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G43" r:id="R29b62d037c264986"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G44" r:id="R0e2fde9e41914bc0"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G45" r:id="R8a6f7c1c240b4984"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G46" r:id="Rc2c8760718ee4052"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G47" r:id="Red864c4f27dd4612"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G48" r:id="R14bf999c7e0549b9"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G49" r:id="R95a4798291074feb"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G50" r:id="R6e3bc7c025c44568"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G51" r:id="R8264e72b01864b3c"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G52" r:id="R7f746086e9c9454d"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G53" r:id="R9d890a3a03d84536"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G54" r:id="Rc3bf21da6fb24482"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G55" r:id="Rdf529216bf0e4cbf"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G56" r:id="R6655e92469704159"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G57" r:id="R04068e482b2c45e0"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G58" r:id="R40408af56eda415b"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G59" r:id="Ra0603fa82f404dcc"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G60" r:id="Rce8d385bd33745fa"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G61" r:id="R77e76054c6ed44f7"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G62" r:id="R727e3bba0c5749a4"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G63" r:id="R4a398e02ed224b40"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G64" r:id="Rfae50000d1b24632"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G65" r:id="R50ed42ab9a2e40a4"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G66" r:id="R23d2c7d2f9d144cf"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G67" r:id="R9e7dd4a1a5694ad2"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G68" r:id="rId1"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G69" r:id="rId2"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G70" r:id="rId3"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G4" r:id="R5fe9149a74fa466b"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G5" r:id="Rc7bebf68ad284fe9"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G6" r:id="R1da9f95afedd4382"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G7" r:id="R5fc2bb5b32954abe"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G8" r:id="Rd4dc6a88278242df"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G9" r:id="Rc2e28d54204c4e04"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G10" r:id="R7efbfd984dbc4331"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G11" r:id="R426f8da6035b4969"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G12" r:id="R4222a477273e4063"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G13" r:id="R5afc6803f022429f"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G14" r:id="R646e7974b5fb451c"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G15" r:id="R9aa8dae89f92444c"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G16" r:id="R47106c02f8ce4e44"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G17" r:id="R4bb2243994904cd5"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G18" r:id="R4878c60c349e4f53"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G19" r:id="R182a089f569943b6"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G20" r:id="R125d6266b36b4294"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G21" r:id="Ra09b551750454708"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G22" r:id="Rd59aeef03f414f8a"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G23" r:id="Rd7efdbf54c954837"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G24" r:id="R009ed0df9fc6469a"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G25" r:id="R29abdae9e2bd47ed"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G26" r:id="R924c6270904e42e6"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G27" r:id="R12bb1bb6fdd14061"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G28" r:id="R7dc9a8c2631145db"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G29" r:id="Ra14af32ef7594eba"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G30" r:id="R002f6dd1467b4282"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G31" r:id="Reca472297d724495"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G32" r:id="R3fbdb99300984915"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G33" r:id="R95f864f75f4446c5"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G34" r:id="R854c32fd0bd141c4"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G35" r:id="R801cdf73d2ac4035"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G36" r:id="R3365317d0a0840e9"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G37" r:id="R619177f7c3af479d"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G38" r:id="Re9c91d2701224091"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G39" r:id="R7f6c3a353b0e4307"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G40" r:id="Rc9e6863835f54d8c"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G41" r:id="Rf3ec1b2ea608472c"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G42" r:id="R7087c882fe724e98"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G43" r:id="R283948996a7b4196"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G44" r:id="Rad90764a6fa44bbb"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G45" r:id="Rd322c13565604dc2"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G46" r:id="R57021a0ae80f46df"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G47" r:id="R81ac8b11b2e34115"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G48" r:id="Re7643da2d24e4799"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G49" r:id="R11d88e82d3e24882"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G50" r:id="R628701db232043b0"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G51" r:id="R58293887ad5a42a5"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G52" r:id="R8582731c02d44d09"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G53" r:id="R8500f9f883ca4b93"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G54" r:id="Rb4c46518af524795"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G55" r:id="R08568c5d4adb4a18"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G56" r:id="R28064b63025f4d01"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G57" r:id="R50a11ce13d444469"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G58" r:id="Rd4813e4d3d40423d"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G59" r:id="Ra1076960becd4ff4"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G60" r:id="R26802b140be94641"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G61" r:id="Rd923e46eb0ee401f"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G62" r:id="R1f1f436dc81f49a6"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G63" r:id="R5ef82cafc686493f"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G64" r:id="R2d20f8f00bb04da8"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G65" r:id="R47eadf9e54344225"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G66" r:id="R31d449955f874e27"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G67" r:id="R9e6f6d6596264c92"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G68" r:id="Rd81b542e40dd464e"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G69" r:id="R1d656746da874844"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G70" r:id="R9f4a842dc68d43a7"/>
   </x:hyperlinks>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb66a9df849a34148"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2716d246c52b43cb"/>
 </x:worksheet>
 </file>
</xml_diff>